<commit_message>
test: align growth history with review dates
</commit_message>
<xml_diff>
--- a/public/test-data/00_성과평가_빠른시작_통합_테스트.xlsx
+++ b/public/test-data/00_성과평가_빠른시작_통합_테스트.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="빠른시작 안내" sheetId="1" r:id="R29a7c328eb224470"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="과제양식" sheetId="2" r:id="R5198400516cf43be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="팀원양식" sheetId="3" r:id="R4b80bcd67c484706"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="성과입력" sheetId="4" r:id="R08e893e090c84f26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="피어리뷰" sheetId="5" r:id="Rd1fde30cd3a3444a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="빠른시작 안내" sheetId="1" r:id="R2f512f01ae2848a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="과제양식" sheetId="2" r:id="R2a314d69b30c41de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="팀원양식" sheetId="3" r:id="Ra7b341ab796a468e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="성과입력" sheetId="4" r:id="R3cd1d47c5f3b4540"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="피어리뷰" sheetId="5" r:id="R2a3e2b98e9b54863"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -702,7 +702,7 @@
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
       <x:c r="A2" s="22" t="str">
-        <x:v>팀원 5명 · 2021~2025년 업적(상/하)·역량 이력</x:v>
+        <x:v>팀원별 승진심사 시기 직전 5개년 업적(상/하)·역량 이력</x:v>
       </x:c>
       <x:c r="B2" s="22"/>
       <x:c r="C2" s="22"/>
@@ -745,16 +745,16 @@
         <x:v>2029-09</x:v>
       </x:c>
       <x:c r="D5" s="21" t="n">
-        <x:v>2025</x:v>
+        <x:v>2028</x:v>
       </x:c>
       <x:c r="E5" s="28" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F5" s="28" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="F5" s="28" t="str">
-        <x:v>A</x:v>
-      </x:c>
       <x:c r="G5" s="28" t="str">
-        <x:v>S</x:v>
+        <x:v>A</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="21" customHeight="1">
@@ -762,16 +762,16 @@
       <x:c r="B6" s="29" t="str"/>
       <x:c r="C6" s="29" t="str"/>
       <x:c r="D6" s="21" t="n">
-        <x:v>2024</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E6" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>S</x:v>
       </x:c>
       <x:c r="F6" s="28" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="G6" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="21" customHeight="1">
@@ -779,7 +779,7 @@
       <x:c r="B7" s="29" t="str"/>
       <x:c r="C7" s="29" t="str"/>
       <x:c r="D7" s="21" t="n">
-        <x:v>2023</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E7" s="28" t="str">
         <x:v>B</x:v>
@@ -788,7 +788,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="G7" s="28" t="str">
-        <x:v>S</x:v>
+        <x:v>B</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="21" customHeight="1">
@@ -796,16 +796,16 @@
       <x:c r="B8" s="29" t="str"/>
       <x:c r="C8" s="29" t="str"/>
       <x:c r="D8" s="21" t="n">
-        <x:v>2022</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="E8" s="28" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="F8" s="28" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="F8" s="28" t="str">
-        <x:v>B</x:v>
-      </x:c>
       <x:c r="G8" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="21" customHeight="1">
@@ -813,16 +813,16 @@
       <x:c r="B9" s="29" t="str"/>
       <x:c r="C9" s="29" t="str"/>
       <x:c r="D9" s="21" t="n">
-        <x:v>2021</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="E9" s="28" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F9" s="28" t="str">
         <x:v>S</x:v>
       </x:c>
-      <x:c r="F9" s="28" t="str">
-        <x:v>B</x:v>
-      </x:c>
       <x:c r="G9" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="21" customHeight="1">
@@ -836,16 +836,16 @@
         <x:v>2029-04</x:v>
       </x:c>
       <x:c r="D10" s="21" t="n">
-        <x:v>2025</x:v>
+        <x:v>2028</x:v>
       </x:c>
       <x:c r="E10" s="28" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="F10" s="28" t="str">
-        <x:v>S</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="G10" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="21" customHeight="1">
@@ -853,16 +853,16 @@
       <x:c r="B11" s="29" t="str"/>
       <x:c r="C11" s="29" t="str"/>
       <x:c r="D11" s="21" t="n">
-        <x:v>2024</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E11" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>S</x:v>
       </x:c>
       <x:c r="F11" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="G11" s="28" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="21" customHeight="1">
@@ -870,16 +870,16 @@
       <x:c r="B12" s="29" t="str"/>
       <x:c r="C12" s="29" t="str"/>
       <x:c r="D12" s="21" t="n">
-        <x:v>2023</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E12" s="28" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="F12" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="G12" s="28" t="str">
-        <x:v>S</x:v>
+        <x:v>A</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="21" customHeight="1">
@@ -887,16 +887,16 @@
       <x:c r="B13" s="29" t="str"/>
       <x:c r="C13" s="29" t="str"/>
       <x:c r="D13" s="21" t="n">
-        <x:v>2022</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="E13" s="28" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F13" s="28" t="str">
         <x:v>S</x:v>
       </x:c>
-      <x:c r="F13" s="28" t="str">
-        <x:v>A</x:v>
-      </x:c>
       <x:c r="G13" s="28" t="str">
-        <x:v>C</x:v>
+        <x:v>S</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="21" customHeight="1">
@@ -904,16 +904,16 @@
       <x:c r="B14" s="29" t="str"/>
       <x:c r="C14" s="29" t="str"/>
       <x:c r="D14" s="21" t="n">
-        <x:v>2021</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="E14" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="F14" s="28" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="G14" s="28" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="21" customHeight="1">
@@ -927,13 +927,13 @@
         <x:v>2029-05</x:v>
       </x:c>
       <x:c r="D15" s="21" t="n">
-        <x:v>2025</x:v>
+        <x:v>2028</x:v>
       </x:c>
       <x:c r="E15" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="F15" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="G15" s="28" t="str">
         <x:v>A</x:v>
@@ -944,16 +944,16 @@
       <x:c r="B16" s="29" t="str"/>
       <x:c r="C16" s="29" t="str"/>
       <x:c r="D16" s="21" t="n">
-        <x:v>2024</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E16" s="28" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="F16" s="28" t="str">
-        <x:v>S</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="G16" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="21" customHeight="1">
@@ -961,16 +961,16 @@
       <x:c r="B17" s="29" t="str"/>
       <x:c r="C17" s="29" t="str"/>
       <x:c r="D17" s="21" t="n">
-        <x:v>2023</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E17" s="28" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="F17" s="28" t="str">
-        <x:v>C</x:v>
+        <x:v>S</x:v>
       </x:c>
       <x:c r="G17" s="28" t="str">
-        <x:v>D</x:v>
+        <x:v>B</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="21" customHeight="1">
@@ -978,16 +978,16 @@
       <x:c r="B18" s="29" t="str"/>
       <x:c r="C18" s="29" t="str"/>
       <x:c r="D18" s="21" t="n">
-        <x:v>2022</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="E18" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F18" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="G18" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>D</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="21" customHeight="1">
@@ -995,16 +995,16 @@
       <x:c r="B19" s="29" t="str"/>
       <x:c r="C19" s="29" t="str"/>
       <x:c r="D19" s="21" t="n">
-        <x:v>2021</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="E19" s="28" t="str">
-        <x:v>D</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="F19" s="28" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="G19" s="28" t="str">
-        <x:v>D</x:v>
+        <x:v>A</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="21" customHeight="1">
@@ -1018,16 +1018,16 @@
         <x:v>2029-04</x:v>
       </x:c>
       <x:c r="D20" s="21" t="n">
-        <x:v>2025</x:v>
+        <x:v>2028</x:v>
       </x:c>
       <x:c r="E20" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="F20" s="28" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="G20" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>D</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="21" customHeight="1">
@@ -1035,16 +1035,16 @@
       <x:c r="B21" s="29" t="str"/>
       <x:c r="C21" s="29" t="str"/>
       <x:c r="D21" s="21" t="n">
-        <x:v>2024</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E21" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="F21" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="G21" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="21" customHeight="1">
@@ -1052,10 +1052,10 @@
       <x:c r="B22" s="29" t="str"/>
       <x:c r="C22" s="29" t="str"/>
       <x:c r="D22" s="21" t="n">
-        <x:v>2023</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E22" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F22" s="28" t="str">
         <x:v>B</x:v>
@@ -1069,16 +1069,16 @@
       <x:c r="B23" s="29" t="str"/>
       <x:c r="C23" s="29" t="str"/>
       <x:c r="D23" s="21" t="n">
-        <x:v>2022</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="E23" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F23" s="28" t="str">
-        <x:v>S</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="G23" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="21" customHeight="1">
@@ -1086,16 +1086,16 @@
       <x:c r="B24" s="29" t="str"/>
       <x:c r="C24" s="29" t="str"/>
       <x:c r="D24" s="21" t="n">
-        <x:v>2021</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="E24" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="F24" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="G24" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>S</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="21" customHeight="1">
@@ -1109,7 +1109,7 @@
         <x:v>2029-03</x:v>
       </x:c>
       <x:c r="D25" s="21" t="n">
-        <x:v>2025</x:v>
+        <x:v>2028</x:v>
       </x:c>
       <x:c r="E25" s="28" t="str">
         <x:v>A</x:v>
@@ -1126,16 +1126,16 @@
       <x:c r="B26" s="29" t="str"/>
       <x:c r="C26" s="29" t="str"/>
       <x:c r="D26" s="21" t="n">
-        <x:v>2024</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E26" s="28" t="str">
-        <x:v>D</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F26" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="G26" s="28" t="str">
-        <x:v>C</x:v>
+        <x:v>A</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="21" customHeight="1">
@@ -1143,16 +1143,16 @@
       <x:c r="B27" s="29" t="str"/>
       <x:c r="C27" s="29" t="str"/>
       <x:c r="D27" s="21" t="n">
-        <x:v>2023</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E27" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F27" s="28" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="G27" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>D</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="21" customHeight="1">
@@ -1160,16 +1160,16 @@
       <x:c r="B28" s="29" t="str"/>
       <x:c r="C28" s="29" t="str"/>
       <x:c r="D28" s="21" t="n">
-        <x:v>2022</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="E28" s="28" t="str">
-        <x:v>S</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F28" s="28" t="str">
-        <x:v>S</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="G28" s="28" t="str">
-        <x:v>C</x:v>
+        <x:v>A</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="21" customHeight="1">
@@ -1177,16 +1177,16 @@
       <x:c r="B29" s="29" t="str"/>
       <x:c r="C29" s="29" t="str"/>
       <x:c r="D29" s="21" t="n">
-        <x:v>2021</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="E29" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="F29" s="28" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="G29" s="28" t="str">
-        <x:v>B</x:v>
+        <x:v>S</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>